<commit_message>
The modified density by depth from March 2026 is the Claude version of the error bar plot. Need to fix up differences and proportion in the original script
</commit_message>
<xml_diff>
--- a/PostWasting_PreWasting_Differences_20260117.xlsx
+++ b/PostWasting_PreWasting_Differences_20260117.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alyssaplayer/Desktop/AP-VRG-PVR-RefugiaAR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646B0C99-186B-574B-A56E-56CEED19F8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8290D994-3D8D-974B-AA1C-F2E19FF802FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15140" yWindow="680" windowWidth="15120" windowHeight="17340" xr2:uid="{2B88350A-688B-394D-9B31-73924C2CF7D3}"/>
+    <workbookView xWindow="15120" yWindow="660" windowWidth="15120" windowHeight="17200" xr2:uid="{2B88350A-688B-394D-9B31-73924C2CF7D3}"/>
   </bookViews>
   <sheets>
     <sheet name="PostWasting_PreWasting_Differen" sheetId="1" r:id="rId1"/>
@@ -105,7 +105,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1059,7 +1059,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC53CF96-F6F3-9C4C-8774-D459D1529388}">
   <dimension ref="A1:M21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
     <col min="2" max="2" width="19.83203125" customWidth="1"/>
@@ -1073,7 +1073,7 @@
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="17" thickBot="1">
+    <row r="1" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>4.1003346262239306</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>0.86867234061038734</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>0.60004621195151886</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="17" thickBot="1">
+    <row r="5" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>14</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>0.64217027713580255</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>2.7418028541750119</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>0.86044104765949836</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>0.72100018799689991</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="17" thickBot="1">
+    <row r="9" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>13</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>0.72522334731777482</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>14.096085346092528</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>3.5274261528265223</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>13</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>5.3168949759707029</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="17" thickBot="1">
+    <row r="13" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>14</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>5.5724760297159612</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="M14" s="6"/>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>13</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>1.8273142244605758</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>12</v>
       </c>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="M16" s="11"/>
     </row>
-    <row r="17" spans="1:13" ht="17" thickBot="1">
+    <row r="17" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>14</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>0.18204095725128774</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>2.0748838891730612</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>13</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>0.58064696416498829</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>12</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>0.43307390590266048</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="17" thickBot="1">
+    <row r="21" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>14</v>
       </c>

</xml_diff>